<commit_message>
Add Word doc + Change-vs-Baseline analysis to August D2C plan
- Word doc (.docx) with full plan and June->August change narrative
- New Excel tab "6. Change vs Baseline": segment + category deltas
- Quantifies additional new/repeat orders & users, cost, and source categories
  vs the June baseline (+599 new, +4,664 repeat orders; ~+Rs19L Meta spend)

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01En7p7RwqiQmLEi9QPf4oKA
</commit_message>
<xml_diff>
--- a/august-d2c-plan/DailyObjects_August_D2C_Plan.xlsx
+++ b/august-d2c-plan/DailyObjects_August_D2C_Plan.xlsx
@@ -1,17 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="1. Exec Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="2. New vs Repeat" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="3. Category Targets" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="4. Meta Baseline" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="5. Weekend Freebie" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1. Exec Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2. New vs Repeat" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3. Category Targets" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4. Meta Baseline" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5. Weekend Freebie" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6. Change vs Baseline" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -20,14 +21,17 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="5">
+  <numFmts count="8">
     <numFmt numFmtId="164" formatCode="&quot;₹&quot;#,##0"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
     <numFmt numFmtId="166" formatCode="&quot;₹&quot;#,##0.00&quot; cr&quot;"/>
     <numFmt numFmtId="167" formatCode="0.00&quot;x&quot;"/>
     <numFmt numFmtId="168" formatCode="&quot;₹&quot;#,##0.0&quot; L&quot;"/>
+    <numFmt numFmtId="169" formatCode="+#,##0;-#,##0"/>
+    <numFmt numFmtId="170" formatCode="+0.0%;-0.0%"/>
+    <numFmt numFmtId="171" formatCode="&quot;₹&quot;+#,##0;&quot;₹&quot;-#,##0"/>
   </numFmts>
-  <fonts count="15">
+  <fonts count="18">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -113,6 +117,21 @@
       <color rgb="00FFFFFF"/>
       <sz val="9"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="001F2A44"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="00333333"/>
+      <sz val="9"/>
+    </font>
   </fonts>
   <fills count="9">
     <fill>
@@ -157,7 +176,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -179,11 +198,55 @@
         <color rgb="00C9C9C9"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00C9C9C9"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00C9C9C9"/>
+      </right>
+      <top style="thin">
+        <color rgb="00C9C9C9"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00C9C9C9"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00C9C9C9"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00C9C9C9"/>
+      </right>
+      <top style="thin">
+        <color rgb="00C9C9C9"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00C9C9C9"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="77">
+  <cellXfs count="119">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -412,6 +475,128 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="170" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="170" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="11" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="11" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="170" fontId="11" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="13" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="171" fontId="13" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="13" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="171" fontId="13" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="13" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="171" fontId="13" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="13" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="171" fontId="13" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="14" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="171" fontId="14" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1124,6 +1309,11 @@
           <t>1.  New users: 2.97 M  →  18,762 new orders. Concentrate spend on Power Bank, Stack, Node (ROAS &gt;3.15, high/med LTV).</t>
         </is>
       </c>
+      <c r="B17" s="77" t="n"/>
+      <c r="C17" s="77" t="n"/>
+      <c r="D17" s="77" t="n"/>
+      <c r="E17" s="77" t="n"/>
+      <c r="F17" s="78" t="n"/>
     </row>
     <row r="18" ht="30" customHeight="1">
       <c r="A18" s="12" t="inlineStr">
@@ -1131,6 +1321,11 @@
           <t>2.  Repeat users: 1.43 M  →  21,864 repeat orders. Drive via CRM + app push + retargeting; freebie weekends reactivate.</t>
         </is>
       </c>
+      <c r="B18" s="77" t="n"/>
+      <c r="C18" s="77" t="n"/>
+      <c r="D18" s="77" t="n"/>
+      <c r="E18" s="77" t="n"/>
+      <c r="F18" s="78" t="n"/>
     </row>
     <row r="19" ht="30" customHeight="1">
       <c r="A19" s="12" t="inlineStr">
@@ -1138,6 +1333,11 @@
           <t>3.  Mix goal: 46% new / 54% repeat orders (was 54/46) — shifts blend to efficiency without losing topline.</t>
         </is>
       </c>
+      <c r="B19" s="77" t="n"/>
+      <c r="C19" s="77" t="n"/>
+      <c r="D19" s="77" t="n"/>
+      <c r="E19" s="77" t="n"/>
+      <c r="F19" s="78" t="n"/>
     </row>
     <row r="20" ht="30" customHeight="1">
       <c r="A20" s="12" t="inlineStr">
@@ -1145,6 +1345,11 @@
           <t>4.  Hold blended Meta ROAS ≥ 3.28x (last-4-day bar); plan lands 3.39x.</t>
         </is>
       </c>
+      <c r="B20" s="77" t="n"/>
+      <c r="C20" s="77" t="n"/>
+      <c r="D20" s="77" t="n"/>
+      <c r="E20" s="77" t="n"/>
+      <c r="F20" s="78" t="n"/>
     </row>
     <row r="21" ht="30" customHeight="1">
       <c r="A21" s="12" t="inlineStr">
@@ -1152,6 +1357,11 @@
           <t>5.  4 freebie weekends add ~₹0.38 cr incremental at accretive ROAS (see tab 5).</t>
         </is>
       </c>
+      <c r="B21" s="77" t="n"/>
+      <c r="C21" s="77" t="n"/>
+      <c r="D21" s="77" t="n"/>
+      <c r="E21" s="77" t="n"/>
+      <c r="F21" s="78" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="7">
@@ -2757,4 +2967,630 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J27"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="23" customWidth="1" min="1" max="1"/>
+    <col width="7" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="79" t="inlineStr">
+        <is>
+          <t>Change vs Baseline — June 2026 → August 2026 target</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="80" t="inlineStr">
+        <is>
+          <t>June is the stated baseline month. Shows the shift needed: how many additional new/repeat orders &amp; users, at what cost, from which categories.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="81" t="inlineStr">
+        <is>
+          <t>SEGMENT CHANGE (D2C, web+app)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="24" t="inlineStr">
+        <is>
+          <t>Segment</t>
+        </is>
+      </c>
+      <c r="B5" s="25" t="inlineStr">
+        <is>
+          <t>June actual</t>
+        </is>
+      </c>
+      <c r="C5" s="25" t="inlineStr">
+        <is>
+          <t>August target</t>
+        </is>
+      </c>
+      <c r="D5" s="25" t="inlineStr">
+        <is>
+          <t>Δ orders</t>
+        </is>
+      </c>
+      <c r="E5" s="25" t="inlineStr">
+        <is>
+          <t>Δ %</t>
+        </is>
+      </c>
+      <c r="F5" s="25" t="inlineStr">
+        <is>
+          <t>Δ users (at plan CVR)</t>
+        </is>
+      </c>
+      <c r="G5" s="24" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="82" t="inlineStr">
+        <is>
+          <t>New orders</t>
+        </is>
+      </c>
+      <c r="B6" s="83" t="n">
+        <v>18163</v>
+      </c>
+      <c r="C6" s="83" t="n">
+        <v>18762</v>
+      </c>
+      <c r="D6" s="84" t="n">
+        <v>599</v>
+      </c>
+      <c r="E6" s="85" t="n">
+        <v>0.03297913340307224</v>
+      </c>
+      <c r="F6" s="84" t="n">
+        <v>-965590</v>
+      </c>
+      <c r="G6" s="19" t="inlineStr">
+        <is>
+          <t>Sessions FALL: new CVR normalises 0.46%→0.63%</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="86" t="inlineStr">
+        <is>
+          <t>Repeat orders</t>
+        </is>
+      </c>
+      <c r="B7" s="87" t="n">
+        <v>17200</v>
+      </c>
+      <c r="C7" s="87" t="n">
+        <v>21864</v>
+      </c>
+      <c r="D7" s="88" t="n">
+        <v>4664</v>
+      </c>
+      <c r="E7" s="89" t="n">
+        <v>0.2711627906976743</v>
+      </c>
+      <c r="F7" s="88" t="n">
+        <v>363898</v>
+      </c>
+      <c r="G7" s="15" t="inlineStr">
+        <is>
+          <t>The real volume engine for August</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="90" t="inlineStr">
+        <is>
+          <t>TOTAL orders</t>
+        </is>
+      </c>
+      <c r="B8" s="91" t="n">
+        <v>35363</v>
+      </c>
+      <c r="C8" s="91" t="n">
+        <v>40626</v>
+      </c>
+      <c r="D8" s="92" t="n">
+        <v>5263</v>
+      </c>
+      <c r="E8" s="93" t="n">
+        <v>0.1488278709385515</v>
+      </c>
+      <c r="F8" s="92" t="n">
+        <v>-601692</v>
+      </c>
+      <c r="G8" s="94" t="inlineStr"/>
+    </row>
+    <row r="10" ht="30" customHeight="1">
+      <c r="A10" s="95" t="inlineStr">
+        <is>
+          <t>Revenue: ₹9.09 cr → ₹10.50 cr  (+₹1.41 cr, +15.5%). ~₹1.26 cr of the +₹1.41 cr comes from repeat. Incremental Meta spend to fund the shift ≈ ₹19 L.</t>
+        </is>
+      </c>
+      <c r="B10" s="77" t="n"/>
+      <c r="C10" s="77" t="n"/>
+      <c r="D10" s="77" t="n"/>
+      <c r="E10" s="77" t="n"/>
+      <c r="F10" s="77" t="n"/>
+      <c r="G10" s="78" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="81" t="inlineStr">
+        <is>
+          <t>CATEGORY CHANGE — where the additional orders &amp; users come from</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="96" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="B13" s="96" t="inlineStr">
+        <is>
+          <t>LTV</t>
+        </is>
+      </c>
+      <c r="C13" s="97" t="inlineStr">
+        <is>
+          <t>New Jun→Aug</t>
+        </is>
+      </c>
+      <c r="D13" s="97" t="inlineStr">
+        <is>
+          <t>Δ New ord</t>
+        </is>
+      </c>
+      <c r="E13" s="97" t="inlineStr">
+        <is>
+          <t>Δ New users</t>
+        </is>
+      </c>
+      <c r="F13" s="97" t="inlineStr">
+        <is>
+          <t>Repeat Jun→Aug</t>
+        </is>
+      </c>
+      <c r="G13" s="97" t="inlineStr">
+        <is>
+          <t>Δ Rep ord</t>
+        </is>
+      </c>
+      <c r="H13" s="97" t="inlineStr">
+        <is>
+          <t>Δ Rep users</t>
+        </is>
+      </c>
+      <c r="I13" s="97" t="inlineStr">
+        <is>
+          <t>Δ Spend New</t>
+        </is>
+      </c>
+      <c r="J13" s="97" t="inlineStr">
+        <is>
+          <t>Δ Spend Rep</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="98" t="inlineStr">
+        <is>
+          <t>Stack</t>
+        </is>
+      </c>
+      <c r="B14" s="99" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="C14" s="99" t="inlineStr">
+        <is>
+          <t>4,453 → 4,957</t>
+        </is>
+      </c>
+      <c r="D14" s="100" t="n">
+        <v>503</v>
+      </c>
+      <c r="E14" s="100" t="n">
+        <v>79654</v>
+      </c>
+      <c r="F14" s="99" t="inlineStr">
+        <is>
+          <t>4,217 → 6,255</t>
+        </is>
+      </c>
+      <c r="G14" s="100" t="n">
+        <v>2038</v>
+      </c>
+      <c r="H14" s="100" t="n">
+        <v>133283</v>
+      </c>
+      <c r="I14" s="101" t="n">
+        <v>399983</v>
+      </c>
+      <c r="J14" s="101" t="n">
+        <v>616972</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="98" t="inlineStr">
+        <is>
+          <t>Power Bank</t>
+        </is>
+      </c>
+      <c r="B15" s="99" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="C15" s="99" t="inlineStr">
+        <is>
+          <t>3,424 → 3,812</t>
+        </is>
+      </c>
+      <c r="D15" s="100" t="n">
+        <v>387</v>
+      </c>
+      <c r="E15" s="100" t="n">
+        <v>61249</v>
+      </c>
+      <c r="F15" s="99" t="inlineStr">
+        <is>
+          <t>3,243 → 4,810</t>
+        </is>
+      </c>
+      <c r="G15" s="100" t="n">
+        <v>1567</v>
+      </c>
+      <c r="H15" s="100" t="n">
+        <v>102486</v>
+      </c>
+      <c r="I15" s="101" t="n">
+        <v>394685</v>
+      </c>
+      <c r="J15" s="101" t="n">
+        <v>474412</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="102" t="inlineStr">
+        <is>
+          <t>Node</t>
+        </is>
+      </c>
+      <c r="B16" s="103" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="C16" s="103" t="inlineStr">
+        <is>
+          <t>2,766 → 2,677</t>
+        </is>
+      </c>
+      <c r="D16" s="104" t="n">
+        <v>-89</v>
+      </c>
+      <c r="E16" s="104" t="n">
+        <v>-14064</v>
+      </c>
+      <c r="F16" s="103" t="inlineStr">
+        <is>
+          <t>2,619 → 2,877</t>
+        </is>
+      </c>
+      <c r="G16" s="104" t="n">
+        <v>258</v>
+      </c>
+      <c r="H16" s="104" t="n">
+        <v>16902</v>
+      </c>
+      <c r="I16" s="105" t="n">
+        <v>-121988</v>
+      </c>
+      <c r="J16" s="105" t="n">
+        <v>78240</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="106" t="inlineStr">
+        <is>
+          <t>Tech Kit (Park)</t>
+        </is>
+      </c>
+      <c r="B17" s="107" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="C17" s="107" t="inlineStr">
+        <is>
+          <t>2,283 → 2,209</t>
+        </is>
+      </c>
+      <c r="D17" s="108" t="n">
+        <v>-73</v>
+      </c>
+      <c r="E17" s="108" t="n">
+        <v>-11608</v>
+      </c>
+      <c r="F17" s="107" t="inlineStr">
+        <is>
+          <t>2,161 → 2,375</t>
+        </is>
+      </c>
+      <c r="G17" s="108" t="n">
+        <v>213</v>
+      </c>
+      <c r="H17" s="108" t="n">
+        <v>13950</v>
+      </c>
+      <c r="I17" s="109" t="n">
+        <v>-67832</v>
+      </c>
+      <c r="J17" s="109" t="n">
+        <v>64575</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="102" t="inlineStr">
+        <is>
+          <t>Bags / DG</t>
+        </is>
+      </c>
+      <c r="B18" s="103" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="C18" s="103" t="inlineStr">
+        <is>
+          <t>1,571 → 1,521</t>
+        </is>
+      </c>
+      <c r="D18" s="104" t="n">
+        <v>-50</v>
+      </c>
+      <c r="E18" s="104" t="n">
+        <v>-7990</v>
+      </c>
+      <c r="F18" s="103" t="inlineStr">
+        <is>
+          <t>1,488 → 1,635</t>
+        </is>
+      </c>
+      <c r="G18" s="104" t="n">
+        <v>147</v>
+      </c>
+      <c r="H18" s="104" t="n">
+        <v>9602</v>
+      </c>
+      <c r="I18" s="105" t="n">
+        <v>-42220</v>
+      </c>
+      <c r="J18" s="105" t="n">
+        <v>44449</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="98" t="inlineStr">
+        <is>
+          <t>Charging Station (Loft)</t>
+        </is>
+      </c>
+      <c r="B19" s="99" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="C19" s="99" t="inlineStr">
+        <is>
+          <t>1,310 → 1,458</t>
+        </is>
+      </c>
+      <c r="D19" s="100" t="n">
+        <v>148</v>
+      </c>
+      <c r="E19" s="100" t="n">
+        <v>23429</v>
+      </c>
+      <c r="F19" s="99" t="inlineStr">
+        <is>
+          <t>1,240 → 1,840</t>
+        </is>
+      </c>
+      <c r="G19" s="100" t="n">
+        <v>599</v>
+      </c>
+      <c r="H19" s="100" t="n">
+        <v>39203</v>
+      </c>
+      <c r="I19" s="101" t="n">
+        <v>170215</v>
+      </c>
+      <c r="J19" s="101" t="n">
+        <v>181473</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="102" t="inlineStr">
+        <is>
+          <t>Desk Organiser (Bar)</t>
+        </is>
+      </c>
+      <c r="B20" s="103" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="C20" s="103" t="inlineStr">
+        <is>
+          <t>1,315 → 1,273</t>
+        </is>
+      </c>
+      <c r="D20" s="104" t="n">
+        <v>-42</v>
+      </c>
+      <c r="E20" s="104" t="n">
+        <v>-6688</v>
+      </c>
+      <c r="F20" s="103" t="inlineStr">
+        <is>
+          <t>1,245 → 1,368</t>
+        </is>
+      </c>
+      <c r="G20" s="104" t="n">
+        <v>123</v>
+      </c>
+      <c r="H20" s="104" t="n">
+        <v>8038</v>
+      </c>
+      <c r="I20" s="105" t="n">
+        <v>-40406</v>
+      </c>
+      <c r="J20" s="105" t="n">
+        <v>37208</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="110" t="inlineStr">
+        <is>
+          <t>Watch Bands</t>
+        </is>
+      </c>
+      <c r="B21" s="111" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="C21" s="111" t="inlineStr">
+        <is>
+          <t>1,041 → 856</t>
+        </is>
+      </c>
+      <c r="D21" s="112" t="n">
+        <v>-185</v>
+      </c>
+      <c r="E21" s="112" t="n">
+        <v>-29203</v>
+      </c>
+      <c r="F21" s="111" t="inlineStr">
+        <is>
+          <t>986 → 704</t>
+        </is>
+      </c>
+      <c r="G21" s="112" t="n">
+        <v>-282</v>
+      </c>
+      <c r="H21" s="112" t="n">
+        <v>-18428</v>
+      </c>
+      <c r="I21" s="113" t="n">
+        <v>-199416</v>
+      </c>
+      <c r="J21" s="113" t="n">
+        <v>-85303</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="114" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B22" s="114" t="inlineStr"/>
+      <c r="C22" s="115" t="inlineStr">
+        <is>
+          <t>18,163 → 18,762</t>
+        </is>
+      </c>
+      <c r="D22" s="116" t="n">
+        <v>599</v>
+      </c>
+      <c r="E22" s="116" t="n">
+        <v>94778</v>
+      </c>
+      <c r="F22" s="115" t="inlineStr">
+        <is>
+          <t>17,200 → 21,864</t>
+        </is>
+      </c>
+      <c r="G22" s="116" t="n">
+        <v>4664</v>
+      </c>
+      <c r="H22" s="116" t="n">
+        <v>305036</v>
+      </c>
+      <c r="I22" s="117" t="n">
+        <v>493021</v>
+      </c>
+      <c r="J22" s="117" t="n">
+        <v>1412026</v>
+      </c>
+    </row>
+    <row r="24" ht="16" customHeight="1">
+      <c r="A24" s="118" t="inlineStr">
+        <is>
+          <t>Read: grow HIGH-LTV (Stack, Power Bank, Charging Station) on both new &amp; repeat; hold MED; cut Watch Bands (low LTV/ROAS).</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="16" customHeight="1">
+      <c r="A25" s="118" t="inlineStr">
+        <is>
+          <t>Δ New users / Δ Rep users = additional sessions to acquire for the incremental orders, at plan CVR (new 0.63%, repeat 1.53%).</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="16" customHeight="1">
+      <c r="A26" s="118" t="inlineStr">
+        <is>
+          <t>Δ Spend = incremental Meta media: new = Δord × category CAC; repeat = Δord × 35% paid × ₹865. Net new +₹4.9L, repeat +₹14.1L.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="16" customHeight="1">
+      <c r="A27" s="118" t="inlineStr">
+        <is>
+          <t>Repeat additions run via CRM + app push + retargeting — most of the 1.43M repeat sessions are owned-channel, not paid.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="7">
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A27:J27"/>
+    <mergeCell ref="A26:J26"/>
+    <mergeCell ref="A24:J24"/>
+    <mergeCell ref="A2:J2"/>
+    <mergeCell ref="A25:J25"/>
+    <mergeCell ref="A10:G10"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>